<commit_message>
Resolvendo o problema do sistema com numeros parecidos
</commit_message>
<xml_diff>
--- a/Planilhas/Comparação de Encerrantes2.xlsx
+++ b/Planilhas/Comparação de Encerrantes2.xlsx
@@ -10,25 +10,25 @@
     <sheet name="Page 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Page 1'!$A$1:$F$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Page 1'!$A$1:$F$38</definedName>
   </definedNames>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="45">
   <si>
     <t>Comparação de Encerrantes</t>
   </si>
   <si>
-    <t>Data do Movimento: 09/09/2026</t>
-  </si>
-  <si>
-    <t>11/09/2026 13:09:32</t>
-  </si>
-  <si>
-    <t>Empresa: Posto Petromais 2 - 10568309000217</t>
+    <t>Data do Movimento: 06/10/2026</t>
+  </si>
+  <si>
+    <t>08/10/2026 10:10:39</t>
+  </si>
+  <si>
+    <t>Empresa: Prodoeste - Uberaba</t>
   </si>
   <si>
     <t>Bico</t>
@@ -52,7 +52,7 @@
     <t>2</t>
   </si>
   <si>
-    <t>ETANOL COMUM</t>
+    <t>GASOLINA GRID</t>
   </si>
   <si>
     <t>3</t>
@@ -61,9 +61,15 @@
     <t>4</t>
   </si>
   <si>
+    <t>ETANOL ADITIVADO</t>
+  </si>
+  <si>
     <t>5</t>
   </si>
   <si>
+    <t>DIESEL S-10</t>
+  </si>
+  <si>
     <t>6</t>
   </si>
   <si>
@@ -76,22 +82,73 @@
     <t>9</t>
   </si>
   <si>
-    <t>DIESEL COMUM B S-500</t>
-  </si>
-  <si>
     <t>10</t>
   </si>
   <si>
-    <t>DIESEL COMUM B S-10</t>
-  </si>
-  <si>
-    <t>Total da Diferença da Empresa Posto Petromais 2 - 10568309000217</t>
+    <t>DIESEL S-500</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>DIESEL S-10 ADITIVADO</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>16</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>18</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>ARLA 32</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>Total da Diferença da Empresa Prodoeste - Uberaba</t>
   </si>
   <si>
     <t>Total Geral</t>
   </si>
   <si>
-    <t>Adaptive Business 3.25.04.14 r1016 p827 - Gestão Inteligente de Negócios. (T.E.= 0,515s)</t>
+    <t>Adaptive Business 3.26.02.52 r1116 p931 - Gestão Inteligente de Negócios. (T.E.= 0,563s)</t>
   </si>
   <si>
     <t>Página: 1 de 1</t>
@@ -288,7 +345,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6.09953194944" customWidth="1"/>
@@ -356,14 +413,14 @@
         <v>9</v>
       </c>
       <c r="C6" s="8">
-        <v>326188.31</v>
+        <v>1642420.77</v>
       </c>
       <c r="D6" s="8">
-        <v>326174.716</v>
+        <v>1642405.303</v>
       </c>
       <c r="E6" s="8"/>
       <c r="F6" s="8">
-        <v>13.594</v>
+        <v>15.467</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="11.6352" customHeight="1">
@@ -374,14 +431,14 @@
         <v>11</v>
       </c>
       <c r="C7" s="10">
-        <v>621937.29</v>
+        <v>789879.54</v>
       </c>
       <c r="D7" s="10">
-        <v>621916.864</v>
+        <v>789869.854</v>
       </c>
       <c r="E7" s="10"/>
       <c r="F7" s="10">
-        <v>20.426</v>
+        <v>9.686</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="11.6352" customHeight="1">
@@ -392,14 +449,14 @@
         <v>9</v>
       </c>
       <c r="C8" s="8">
-        <v>415913.73</v>
+        <v>2225739.56</v>
       </c>
       <c r="D8" s="8">
-        <v>415899.874</v>
+        <v>2225708.373</v>
       </c>
       <c r="E8" s="8"/>
       <c r="F8" s="8">
-        <v>13.856</v>
+        <v>31.187</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="11.6352" customHeight="1">
@@ -407,177 +464,464 @@
         <v>13</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C9" s="10">
-        <v>832601.06</v>
+        <v>3039447.18</v>
       </c>
       <c r="D9" s="10">
-        <v>832580.331</v>
+        <v>3039406.193</v>
       </c>
       <c r="E9" s="10"/>
       <c r="F9" s="10">
-        <v>20.729</v>
+        <v>40.987</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="10.908" customHeight="1">
       <c r="A10" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="C10" s="8">
-        <v>546586.63</v>
+        <v>3530081.95</v>
       </c>
       <c r="D10" s="8">
-        <v>546569.698</v>
+        <v>3530067.775</v>
       </c>
       <c r="E10" s="8"/>
       <c r="F10" s="8">
-        <v>16.932</v>
+        <v>14.175</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A11" s="5" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C11" s="10">
-        <v>1093205.26</v>
+        <v>2211893.7</v>
       </c>
       <c r="D11" s="10">
-        <v>1093173.387</v>
+        <v>2211620.127</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="10">
-        <v>31.873</v>
+        <v>273.573</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B12" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>9</v>
-      </c>
       <c r="C12" s="8">
-        <v>595684.3</v>
+        <v>5398034.14</v>
       </c>
       <c r="D12" s="8">
-        <v>595667.518</v>
+        <v>5398015.945</v>
       </c>
       <c r="E12" s="8"/>
       <c r="F12" s="8">
-        <v>16.782</v>
+        <v>18.195</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A13" s="5" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C13" s="10">
-        <v>1206778.45</v>
+        <v>4208587.76</v>
       </c>
       <c r="D13" s="10">
-        <v>1206752.18</v>
+        <v>4209180.666</v>
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="10">
-        <v>26.27</v>
+        <v>-592.906</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="10.908" customHeight="1">
       <c r="A14" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="C14" s="8">
-        <v>2815608.31</v>
+        <v>2046521.91</v>
       </c>
       <c r="D14" s="8">
-        <v>2815607.072</v>
+        <v>2046510.163</v>
       </c>
       <c r="E14" s="8"/>
       <c r="F14" s="8">
-        <v>1.238</v>
+        <v>11.747</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="11.6352" customHeight="1">
       <c r="A15" s="5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C15" s="10">
-        <v>606584.46</v>
+        <v>2355908.48</v>
       </c>
       <c r="D15" s="10">
-        <v>1606582.625</v>
+        <v>2355246.903</v>
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="10">
-        <v>-999998.165</v>
+        <v>661.577</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="11.6352" customHeight="1">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B16" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="B16" s="11"/>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11"/>
-      <c r="E16" s="11"/>
-      <c r="F16" s="12">
-        <v>-999836.465</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="5.8176" customHeight="1"/>
+      <c r="C16" s="8">
+        <v>1280558.53</v>
+      </c>
+      <c r="D16" s="8">
+        <v>1280421.931</v>
+      </c>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8">
+        <v>136.599</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A17" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="10">
+        <v>7223774.5</v>
+      </c>
+      <c r="D17" s="10">
+        <v>7223866.473</v>
+      </c>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10">
+        <v>-91.973</v>
+      </c>
+    </row>
     <row r="18" spans="1:6" ht="10.908" customHeight="1">
-      <c r="A18" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="13"/>
-      <c r="E18" s="13"/>
-      <c r="F18" s="14">
-        <v>-999836.465</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="145.44" customHeight="1"/>
-    <row r="20" spans="1:6" ht="145.44" customHeight="1"/>
-    <row r="21" spans="1:6" ht="142.53119999999998" customHeight="1"/>
-    <row r="22" spans="1:6" ht="142.53119999999998" customHeight="1">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15"/>
+      <c r="A18" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" s="8">
+        <v>528820.88</v>
+      </c>
+      <c r="D18" s="8">
+        <v>528804.888</v>
+      </c>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8">
+        <v>15.992</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A19" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" s="10">
+        <v>303498.49</v>
+      </c>
+      <c r="D19" s="10">
+        <v>303490.221</v>
+      </c>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10">
+        <v>8.269</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A20" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" s="8">
+        <v>4876983.58</v>
+      </c>
+      <c r="D20" s="8">
+        <v>876980.457</v>
+      </c>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8">
+        <v>4000003.123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A21" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" s="10">
+        <v>725383.99</v>
+      </c>
+      <c r="D21" s="10">
+        <v>725383.019</v>
+      </c>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10">
+        <v>0.971</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" ht="10.908" customHeight="1">
+      <c r="A22" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C22" s="8">
+        <v>3644613.28</v>
+      </c>
+      <c r="D22" s="8">
+        <v>3644456.243</v>
+      </c>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8">
+        <v>157.037</v>
+      </c>
     </row>
     <row r="23" spans="1:6" ht="11.6352" customHeight="1">
-      <c r="A23" s="16" t="s">
-        <v>24</v>
-      </c>
-      <c r="B23" s="16"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="17" t="s">
-        <v>25</v>
+      <c r="A23" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B23" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="10">
+        <v>9508994.61</v>
+      </c>
+      <c r="D23" s="10">
+        <v>9508869.847</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10">
+        <v>124.763</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A24" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B24" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="8">
+        <v>7760165.78</v>
+      </c>
+      <c r="D24" s="8">
+        <v>7760038.165</v>
+      </c>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8">
+        <v>127.615</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A25" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B25" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="10">
+        <v>3802068.6</v>
+      </c>
+      <c r="D25" s="10">
+        <v>3802059.751</v>
+      </c>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10">
+        <v>8.849</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="10.908" customHeight="1">
+      <c r="A26" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C26" s="8">
+        <v>1649401</v>
+      </c>
+      <c r="D26" s="8">
+        <v>1649384.263</v>
+      </c>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8">
+        <v>16.737</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A27" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B27" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" s="10">
+        <v>802334.16</v>
+      </c>
+      <c r="D27" s="10">
+        <v>802323.219</v>
+      </c>
+      <c r="E27" s="10"/>
+      <c r="F27" s="10">
+        <v>10.941</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A28" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B28" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" s="8">
+        <v>1983484.32</v>
+      </c>
+      <c r="D28" s="8">
+        <v>1983456.946</v>
+      </c>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8">
+        <v>27.374</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A29" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B29" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="10">
+        <v>2855099.58</v>
+      </c>
+      <c r="D29" s="10">
+        <v>2855056.96</v>
+      </c>
+      <c r="E29" s="10"/>
+      <c r="F29" s="10">
+        <v>42.62</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" ht="10.908" customHeight="1">
+      <c r="A30" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C30" s="8">
+        <v>997584.95</v>
+      </c>
+      <c r="D30" s="8">
+        <v>997555.176</v>
+      </c>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8">
+        <v>29.774</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A31" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B31" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="C31" s="10">
+        <v>452419.21</v>
+      </c>
+      <c r="D31" s="10">
+        <v>452389.373</v>
+      </c>
+      <c r="E31" s="10"/>
+      <c r="F31" s="10">
+        <v>29.837</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A32" s="11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="12">
+        <v>4001132.216</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" ht="5.8176" customHeight="1"/>
+    <row r="34" spans="1:6" ht="10.908" customHeight="1">
+      <c r="A34" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="13"/>
+      <c r="F34" s="14">
+        <v>4001132.216</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="145.44" customHeight="1"/>
+    <row r="36" spans="1:6" ht="123.624" customHeight="1"/>
+    <row r="37" spans="1:6" ht="123.624" customHeight="1">
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15"/>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+    </row>
+    <row r="38" spans="1:6" ht="11.6352" customHeight="1">
+      <c r="A38" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16"/>
+      <c r="D38" s="16"/>
+      <c r="E38" s="16"/>
+      <c r="F38" s="17" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
+  <mergeCells count="35">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="E2:F2"/>
@@ -594,9 +938,25 @@
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="D14:E14"/>
     <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A18:E18"/>
-    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A34:E34"/>
+    <mergeCell ref="A38:E38"/>
   </mergeCells>
   <pageMargins left="0.3937007874015748" right="0.3937007874015748" top="0.3937007874015748" bottom="0.3937007874015748" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" fitToHeight="0"/>

</xml_diff>